<commit_message>
2025-01-15 1.修改訂單資料表 	修改欄位: 		f_totalPrice=>f_totalAmount 		f_shippingMethod INT=>f_shippingOption NVARCHAR(10) 	新增欄位: 		f_originalAmount.f_discountAmount.f_shippingFee
2.修改訂單商品資料表
	修改表名稱:
		t_orderProductStyle=>t_orderItem
	修改欄位:
		f_orderProductStyleId=>f_orderItemId
	刪除欄位:
		f_productStyleId
	新增欄位:
		f_productName.f_style

3.新增運輸方式資料表
	t_shippingOption
	f_shippingOptionId.f_option 貨運方式.f_shippingFee 運費金額.f_freeShipping 免運金額.f_createTime.f_updateTime

4.完成運輸費用設定(不可新增只可修改 預設運輸方式為便利商店跟宅配)

Signed-off-by: Annie <FengMu9966@gmail.com>
</commit_message>
<xml_diff>
--- a/document/ProjectUsing/SqlDataTableNotes/資料表設計.xlsx
+++ b/document/ProjectUsing/SqlDataTableNotes/資料表設計.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12720" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="使用者表" sheetId="8" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="商品表" sheetId="5" r:id="rId4"/>
     <sheet name="交易紀錄表" sheetId="10" r:id="rId5"/>
     <sheet name="備用(淘汰的表)" sheetId="12" r:id="rId6"/>
+    <sheet name="待確認" sheetId="13" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="330">
   <si>
     <t>KEY</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -423,10 +424,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>f_totalPrice</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>f_orderId</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -555,31 +552,11 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>f_amount</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>int</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>金額</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">f_transactionType </t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>nvarchar(10)</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>N</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>ex : 付款, 退款</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -763,10 +740,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>細項分類</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>圖片路徑</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -919,38 +892,34 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
+    <t>f_createTime</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>decimal</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>退貨單狀態 (已確認/取消</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>productImage資料表(t_productImage)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_productImageId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>數據行名稱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>f_productStyleId</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>f_createTime</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>decimal</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>退貨單狀態 (已確認/取消</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>productImage資料表(t_productImage)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_productImageId</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>數據行名稱</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_productStyleId</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>productStyle資料表(t_productStyle)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1083,19 +1052,11 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>f_orderProductStyleId</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>會員表外鍵</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>訂單表外鍵</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>商品子項目 (細項) 表外鍵</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -1177,14 +1138,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>N</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>目前提供 1便利商店; 2:宅配</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>f_state</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -1194,22 +1147,6 @@
   </si>
   <si>
     <t>f_createTime</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>王六仔</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1220,10 +1157,6 @@
     <t>日期時間 (YYMMDD) + 時分秒轉成秒(00000~86399) + 會員碼最末7位(EX:0000001)  UNIQUE有唯一性
   (Ex:250106000010000001 、 250107863990000002)</t>
     <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>orderProductStyle資料表(t_orderProductStyle)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>orderState資料表(t_orderState)</t>
@@ -1236,95 +1169,200 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
+    <t>訂單狀態 ( 1:待確認, 2:待出貨, 3:已出貨, 4:完成, 5:買家未取商品, 6:重新寄回, 7:取消, 8:退貨)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>bigint</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>收件人手機號碼 (國內)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>手機號碼 (國內)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>freight資料表(t_freight)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_freightId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>運輸方式 1:便利商店; 2:宅配</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>運費金額</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_freeShipping</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>免運金額</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_shippingFee</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>細項名稱</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_productId</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>商品外鍵</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_originalAmount</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>原價</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_discountAmount</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_discountedAmount</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>折扣的金額</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>折扣後的金額</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_shippintFee</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>運費</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_totalAmount</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>總金額</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_productName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_orderItemId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>orderItem資料表(t_orderItem)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_originalAmount</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>原始金額  (小數點前8位 小數點後2位)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>折扣後金額  (小數點前8位 小數點後2位)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
     <t>int</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>訂單狀態 ( 1:待確認, 2:待出貨, 3:已出貨, 4:完成, 5:買家未取商品, 6:重新寄回, 7:取消, 8:退貨)</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>bigint</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>收件人手機號碼 (國內)</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>手機號碼 (國內)</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>freight資料表(t_freight)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_freightId</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>運輸方式 1:便利商店; 2:宅配</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>運費金額</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_tagId</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>tag資料表(t_tag)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>nvarchar(5)</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_tagName</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>標籤名字</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>f_freeShipping</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>N</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>免運金額</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>標籤外鍵</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_totalAmount</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>nvarchar(10)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>nvarchar(30)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_discountAmount</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_option</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_shippingOption</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>運輸方式 :便利商店; 宅配</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>運輸方式:便利商店; 宅配</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>生成時間</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>修改運費時間</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>GETDATE()</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_updateTime</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>shippingOption資料表(t_shippingOption)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f_shippingOptionId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>f_shippingFee</t>
     <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>OriginalAmount DECIMAL(10, 2)</t>
-  </si>
-  <si>
-    <t>DiscountAmount DECIMAL(10, 2),</t>
-  </si>
-  <si>
-    <t>DiscountedAmount DECIMAL(10, 2),</t>
-  </si>
-  <si>
-    <t>ShippingFee DECIMAL(10, 2),</t>
-  </si>
-  <si>
-    <t>TotalAmount DECIMAL(10, 2)</t>
   </si>
 </sst>
 </file>
@@ -1486,7 +1524,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1526,20 +1564,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1874,14 +1900,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>238</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1908,7 +1934,7 @@
         <v>59</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
@@ -2034,14 +2060,14 @@
       <c r="F11" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="20"/>
+      <c r="A13" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="16"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -2068,7 +2094,7 @@
         <v>6</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>55</v>
@@ -2096,7 +2122,7 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="3" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -2112,7 +2138,7 @@
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="3" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="G17" s="9"/>
     </row>
@@ -2128,8 +2154,8 @@
         <v>35</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="14" t="s">
-        <v>269</v>
+      <c r="F18" s="13" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -2170,14 +2196,14 @@
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -2204,7 +2230,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
@@ -2238,7 +2264,7 @@
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>27</v>
@@ -2255,17 +2281,17 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="G7" s="8"/>
       <c r="I7">
@@ -2275,46 +2301,46 @@
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="3" t="s">
-        <v>302</v>
+        <v>284</v>
       </c>
       <c r="G8" s="8"/>
       <c r="I8" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="4" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="3" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>33</v>
@@ -2324,13 +2350,13 @@
         <v>34</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>26</v>
@@ -2348,10 +2374,10 @@
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="4" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
@@ -2360,16 +2386,16 @@
         <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="32.4" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>9</v>
@@ -2377,8 +2403,8 @@
       <c r="E13" s="2">
         <v>1</v>
       </c>
-      <c r="F13" s="14" t="s">
-        <v>267</v>
+      <c r="F13" s="13" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -2390,14 +2416,14 @@
       <c r="F14" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="18" t="s">
-        <v>236</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
+      <c r="A17" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="16"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -2424,7 +2450,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
@@ -2461,7 +2487,7 @@
         <v>24</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>21</v>
@@ -2471,16 +2497,16 @@
         <v>28</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>21</v>
@@ -2490,35 +2516,35 @@
         <v>29</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="7"/>
       <c r="B24" s="3" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>9</v>
@@ -2553,7 +2579,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="工作表5"/>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" customWidth="1"/>
@@ -2564,18 +2590,17 @@
     <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="13"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2595,12 +2620,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>88</v>
@@ -2612,14 +2637,13 @@
         <v>47</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>88</v>
@@ -2629,504 +2653,653 @@
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="3" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="64.8" x14ac:dyDescent="0.3">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="64.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="3" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="G5" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="3" t="s">
-        <v>96</v>
+      <c r="F5" s="13" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="32.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="4" t="s">
+        <v>274</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="I6" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="32.4" x14ac:dyDescent="0.3">
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="4" t="s">
-        <v>286</v>
+        <v>99</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>25</v>
+        <v>191</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E7" s="2">
-        <v>1</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>299</v>
-      </c>
-      <c r="G7">
-        <v>0.1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="I8" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="4" t="s">
         <v>103</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>298</v>
+        <v>277</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="G9" s="8"/>
-      <c r="I9" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="4" t="s">
         <v>104</v>
       </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+      <c r="B10" s="3" t="s">
+        <v>311</v>
+      </c>
       <c r="C10" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>101</v>
+        <v>263</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>89</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="I10" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="4" t="s">
-        <v>283</v>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="5"/>
+      <c r="B11" s="3" t="s">
+        <v>318</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>284</v>
+        <v>263</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>89</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="G11" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="32.4" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="4" t="s">
-        <v>255</v>
+        <v>320</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>198</v>
+        <v>316</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>215</v>
+        <v>100</v>
       </c>
       <c r="E12" s="2"/>
-      <c r="F12" s="14" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="F12" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="4" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>184</v>
+        <v>263</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
-      <c r="B14" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2"/>
+      <c r="F14" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="32.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="6"/>
+      <c r="B15" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="6"/>
+      <c r="B16" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="17"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="E16" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="6"/>
+      <c r="B17" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B22" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="F22" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+      <c r="B23" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="3" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
-      <c r="B22" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="G22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
-      <c r="B23" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="B25" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="6"/>
+      <c r="B26" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="6"/>
+      <c r="B27" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="16"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="5"/>
+      <c r="B33" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E33" s="2"/>
+      <c r="F33" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="48.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="5"/>
+      <c r="B34" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="6"/>
+      <c r="B35" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="6"/>
+      <c r="B36" s="4" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="C36" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="6"/>
+      <c r="B37" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="6"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="3"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="14" t="s">
+        <v>327</v>
+      </c>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="16"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E41" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="B42" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="48.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
-      <c r="B30" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="E30" s="2">
-        <v>1</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="6"/>
-      <c r="B31" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" s="3" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="6"/>
-      <c r="B32" s="4" t="s">
+      <c r="F42" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="5"/>
+      <c r="B43" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" s="3" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="6"/>
+      <c r="B44" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
-      <c r="B33" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="6"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="3"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="6"/>
+      <c r="B45" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="6"/>
+      <c r="B46" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="6"/>
+      <c r="B47" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>324</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A26:F26"/>
+  <mergeCells count="4">
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3146,14 +3319,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -3180,17 +3353,17 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="4" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3202,13 +3375,13 @@
         <v>80</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E5" s="2">
         <v>1</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3217,7 +3390,7 @@
         <v>77</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>9</v>
@@ -3233,30 +3406,30 @@
         <v>44</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="3" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="3" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -3274,43 +3447,43 @@
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="3" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F10" s="3" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="B11" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F11" s="3" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -3322,21 +3495,21 @@
       <c r="F12" s="3"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
+      <c r="A14" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>2</v>
@@ -3356,7 +3529,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -3368,7 +3541,7 @@
         <v>8</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -3377,30 +3550,30 @@
         <v>83</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="4" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
       <c r="B18" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="3" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="G18" s="11"/>
       <c r="H18" s="12"/>
@@ -3408,17 +3581,17 @@
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="3" t="s">
-        <v>181</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -3427,14 +3600,14 @@
         <v>79</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="3" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -3450,7 +3623,7 @@
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="3" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -3459,63 +3632,63 @@
         <v>18</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="E22" s="2">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="3" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D23" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F23" s="3" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="7"/>
       <c r="B24" s="3" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F24" s="3" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
+      <c r="A26" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="16"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -3542,7 +3715,7 @@
         <v>6</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>7</v>
@@ -3554,39 +3727,39 @@
         <v>8</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="3" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="4" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
       <c r="B30" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="3" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="G30" s="11"/>
       <c r="H30" s="12"/>
@@ -3614,7 +3787,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="工作表6"/>
-  <dimension ref="A2:H9"/>
+  <dimension ref="A2:H11"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" customWidth="1"/>
@@ -3623,33 +3796,33 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -3657,90 +3830,130 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>124</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
-      <c r="B6" s="3" t="s">
-        <v>129</v>
+      <c r="B6" t="s">
+        <v>296</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>130</v>
+        <v>263</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="3" t="s">
-        <v>131</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="4" t="s">
-        <v>132</v>
+        <v>300</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>133</v>
+        <v>263</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="3" t="s">
-        <v>135</v>
+        <v>301</v>
       </c>
       <c r="H7" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="2"/>
+      <c r="B8" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>299</v>
+      </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>302</v>
+      </c>
       <c r="H8" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="2"/>
+      <c r="B9" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>304</v>
+      </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="6"/>
+      <c r="B10" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3754,7 +3967,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:G36"/>
+  <dimension ref="A2:G30"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" customWidth="1"/>
@@ -3763,14 +3976,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>248</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -3797,7 +4010,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
@@ -3809,13 +4022,13 @@
         <v>8</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>15</v>
@@ -3825,48 +4038,48 @@
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="3" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="3" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="3" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="4" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>25</v>
@@ -3876,55 +4089,55 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="4" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="4" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>82</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="3" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3936,14 +4149,14 @@
       <c r="F12" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>259</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
+      <c r="A14" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -3970,7 +4183,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -3982,13 +4195,13 @@
         <v>8</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="3" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>15</v>
@@ -3998,13 +4211,13 @@
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="3" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="3" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>15</v>
@@ -4014,39 +4227,39 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="3" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="4" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="3" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="3" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -4058,14 +4271,14 @@
       <c r="F21" s="3"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="18" t="s">
-        <v>303</v>
-      </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="20"/>
+      <c r="A23" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -4092,7 +4305,7 @@
         <v>6</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>304</v>
+        <v>286</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>7</v>
@@ -4104,13 +4317,13 @@
         <v>8</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="3" t="s">
-        <v>307</v>
+        <v>294</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>15</v>
@@ -4120,13 +4333,13 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="3" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="4" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>25</v>
@@ -4136,39 +4349,39 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="3" t="s">
-        <v>305</v>
+        <v>287</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
       <c r="B28" s="4" t="s">
-        <v>316</v>
+        <v>292</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="3" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
       <c r="B29" s="4" t="s">
-        <v>312</v>
+        <v>289</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>313</v>
+        <v>290</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="3" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -4179,89 +4392,42 @@
       <c r="E30" s="2"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="18" t="s">
-        <v>308</v>
-      </c>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="20"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="5"/>
-      <c r="B35" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="3" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="5"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="3"/>
-    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A6:B35"/>
+  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="47.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>